<commit_message>
lookup in attribute datasiources invariant of pac cat short notation
</commit_message>
<xml_diff>
--- a/examples/excel_attribute_data.xlsx
+++ b/examples/excel_attribute_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\LabFREED\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{874D1489-ACAE-42D9-9D80-5DACD239FDF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E177F847-C9EE-4C66-A9C4-7E726993E018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67815" yWindow="-4410" windowWidth="32880" windowHeight="19905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="68625" yWindow="180" windowWidth="18420" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>PAC-ID</t>
   </si>
@@ -55,13 +55,22 @@
   </si>
   <si>
     <t>CalibratedWeight</t>
+  </si>
+  <si>
+    <t>HTTPS://PAC.METTORIUS.COM/-MD/BAL500/000001/K:V</t>
+  </si>
+  <si>
+    <t>Anna</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -80,12 +89,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF0451A5"/>
-      <name val="Courier New"/>
-      <family val="3"/>
     </font>
     <font>
       <sz val="11"/>
@@ -125,18 +128,15 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Accent3" xfId="1" builtinId="37"/>
@@ -427,23 +427,23 @@
     <col min="6" max="6" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -468,7 +468,24 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
+      <c r="A3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2">
+        <v>45592</v>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>